<commit_message>
Clarify content import template and guide
</commit_message>
<xml_diff>
--- a/public/content-import-template.xlsx
+++ b/public/content-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Import" sheetId="1" r:id="Rdc75ab72f3524c81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Guide" sheetId="2" r:id="R59245ab26fb24729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Import" sheetId="1" r:id="R2eec8f4203754be4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Guide" sheetId="2" r:id="R6951df436bb643e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -658,9 +658,9 @@
       <x:c r="C1" s="12"/>
       <x:c r="D1" s="12"/>
     </x:row>
-    <x:row r="3" ht="32" customHeight="1">
+    <x:row r="3" ht="44" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Use the Content Import sheet for your data. Its first row is the exact header row expected by Jota.</x:v>
+        <x:v>1. Fill Content Import: keep row 1 unchanged and use one content item per row. 2. Save only that sheet as CSV UTF-8 (comma-delimited). 3. In Jota &gt; Content &gt; Import from CSV, upload it, choose any shared defaults, fix preview errors, then import.</x:v>
       </x:c>
       <x:c r="B3" s="14"/>
       <x:c r="C3" s="14"/>
@@ -668,7 +668,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="str">
-        <x:v>Prompt to copy into an AI tool</x:v>
+        <x:v>Optional AI prompt to copy</x:v>
       </x:c>
       <x:c r="B5" s="16"/>
       <x:c r="C5" s="16"/>
@@ -676,7 +676,10 @@
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="34" t="str">
-        <x:v>Create a UTF-8 CSV for Jota Content Tracker using the exact headers in the Content Import sheet. Create one row for each real content item in the source material I provide. Use only facts from that source; do not invent client, campaign, platform, format, dates, or assigned-person details. Keep client, campaign, and assigned creator/editor names exactly as written in the source. If a required value is missing, ask me instead of guessing. Use dates as YYYY-MM-DD and put the scheduled publishing date under Publish date. Leave optional fields blank when the source does not provide them. If the status is not specified, leave Status blank. Do not include the sample record from the AI Guide sheet, instructions, formulas, extra headings, or commentary in the CSV. Keep the exact headers and order. Quote fields correctly if they contain commas, quotes, or line breaks. Return only the CSV.</x:v>
+        <x:v>Convert the content plan I paste after this prompt into a UTF-8 CSV for Jota. Copy the exact 17 headers from the Content Import sheet in the same order. Make one row per real content item.
+Use only source facts. Do not invent posts, clients, campaigns, platforms, formats, dates, assigned people, workflow statuses, or external client approval. Use exact active Jota names only when I supply them. Repeat the client name in Client / account for every row, even when all rows share one client. Fill Assigned creator / editor with the exact active member name when a supervisor or admin assigns content. Leave Campaign blank for General / Ongoing.
+Every row needs Content title, Platform, and Format. Ask me about missing required details before making the CSV. Use YYYY-MM-DD: Publish date is the posting date, Work date is when production starts, and Deadline is when work is due. Leave unknown optional cells empty; a blank Status becomes Planned.
+Quote commas, quotation marks, and line breaks correctly. Exclude the AI Guide, sample record, formulas, and explanations. Return only the CSV.</x:v>
       </x:c>
       <x:c r="B6" s="35"/>
       <x:c r="C6" s="35"/>
@@ -707,7 +710,7 @@
         <x:v>Client / account</x:v>
       </x:c>
       <x:c r="B11" s="47" t="str">
-        <x:v>Use the exact active client name in Jota. If every row is for one client, this can be left blank and selected as the default during import.</x:v>
+        <x:v>Fill every row with an exact active Jota client name, even when all rows belong to the same client.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
@@ -723,7 +726,7 @@
         <x:v>Required content fields</x:v>
       </x:c>
       <x:c r="B13" s="49" t="str">
-        <x:v>Content title, Platform, and Format must have values. For supervisor/admin imports, also assign a creator/editor or choose one in the import form.</x:v>
+        <x:v>Each row needs Content title, Platform, and Format. Supervisors/admins must also enter the exact active Assigned creator / editor name for that client.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
@@ -731,7 +734,7 @@
         <x:v>Dates</x:v>
       </x:c>
       <x:c r="B14" s="49" t="str">
-        <x:v>Dates are optional. If provided, include the year and use YYYY-MM-DD. Use Publish date for the scheduled posting date.</x:v>
+        <x:v>Dates are optional. Use YYYY-MM-DD with a year: Work date starts production, Deadline is when work is due, and Publish date is the scheduled posting date.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
@@ -747,7 +750,7 @@
         <x:v>Client approval</x:v>
       </x:c>
       <x:c r="B16" s="49" t="str">
-        <x:v>Optional. Use Pending, Approved, Revision Requested, or Rejected.</x:v>
+        <x:v>Optional. Record Pending, Approved, Revision Requested, or Rejected only after a real response through your external client channel. Do not infer approval from status.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
@@ -763,7 +766,7 @@
         <x:v>CSV export</x:v>
       </x:c>
       <x:c r="B18" s="49" t="str">
-        <x:v>Save/export only the Content Import sheet as CSV. Keep its headers in row 1. The sample below is for guidance only; do not import it.</x:v>
+        <x:v>Save only the Content Import sheet as CSV UTF-8 (comma-delimited), not XLSX. Keep headers in row 1; do not include this guide or its sample record.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
@@ -771,7 +774,7 @@
         <x:v>Import limit</x:v>
       </x:c>
       <x:c r="B19" s="51" t="str">
-        <x:v>Jota imports up to 250 content rows at a time. Duplicates are skipped and invalid rows are shown in the preview.</x:v>
+        <x:v>The CSV must be 1 MB or smaller and contain at most 250 content rows. Check the preview: fix invalid rows before importing; duplicates are skipped.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">

</xml_diff>

<commit_message>
Simplify content import template and guidance
</commit_message>
<xml_diff>
--- a/public/content-import-template.xlsx
+++ b/public/content-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Import" sheetId="1" r:id="R2eec8f4203754be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Guide" sheetId="2" r:id="R6951df436bb643e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Import" sheetId="1" r:id="R72329bf4122645ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Guide" sheetId="2" r:id="Rd037121c4a76421d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -59,8 +59,14 @@
       <x:color rgb="FF8C382D"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +93,11 @@
         <x:fgColor rgb="FFFBE9E6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFAD7C43"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="10">
     <x:border>
@@ -191,7 +202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="64">
+  <x:cellXfs count="66">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -336,6 +347,8 @@
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -541,13 +554,13 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
@@ -560,58 +573,38 @@
     <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="9" t="str">
-        <x:v>Client / account</x:v>
-      </x:c>
-      <x:c r="B1" s="9" t="str">
-        <x:v>Campaign</x:v>
-      </x:c>
-      <x:c r="C1" s="9" t="str">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="65" t="str">
         <x:v>Content title</x:v>
       </x:c>
-      <x:c r="D1" s="9" t="str">
+      <x:c r="B1" s="65" t="str">
         <x:v>Platform</x:v>
       </x:c>
-      <x:c r="E1" s="9" t="str">
+      <x:c r="C1" s="65" t="str">
         <x:v>Format</x:v>
       </x:c>
-      <x:c r="F1" s="9" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="G1" s="9" t="str">
+      <x:c r="D1" s="65" t="str">
+        <x:v>Publish date</x:v>
+      </x:c>
+      <x:c r="E1" s="65" t="str">
         <x:v>Work date</x:v>
       </x:c>
-      <x:c r="H1" s="9" t="str">
+      <x:c r="F1" s="65" t="str">
         <x:v>Deadline</x:v>
       </x:c>
-      <x:c r="I1" s="9" t="str">
-        <x:v>Publish date</x:v>
-      </x:c>
-      <x:c r="J1" s="9" t="str">
-        <x:v>Client approval</x:v>
-      </x:c>
-      <x:c r="K1" s="9" t="str">
-        <x:v>Client issues</x:v>
-      </x:c>
-      <x:c r="L1" s="9" t="str">
-        <x:v>Revision count</x:v>
-      </x:c>
-      <x:c r="M1" s="9" t="str">
-        <x:v>Notes / comments</x:v>
-      </x:c>
-      <x:c r="N1" s="9" t="str">
+      <x:c r="G1" s="65" t="str">
         <x:v>Brief / caption</x:v>
       </x:c>
-      <x:c r="O1" s="9" t="str">
-        <x:v>Next action</x:v>
-      </x:c>
-      <x:c r="P1" s="9" t="str">
-        <x:v>Revision feedback</x:v>
-      </x:c>
-      <x:c r="Q1" s="9" t="str">
-        <x:v>Assigned creator / editor</x:v>
-      </x:c>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
+      <x:c r="L1"/>
+      <x:c r="M1"/>
+      <x:c r="N1"/>
+      <x:c r="O1"/>
+      <x:c r="P1"/>
+      <x:c r="Q1"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="10"/>
@@ -652,7 +645,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="12" t="str">
-        <x:v>Content import template</x:v>
+        <x:v>Simple content import</x:v>
       </x:c>
       <x:c r="B1" s="12"/>
       <x:c r="C1" s="12"/>
@@ -660,7 +653,7 @@
     </x:row>
     <x:row r="3" ht="44" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>1. Fill Content Import: keep row 1 unchanged and use one content item per row. 2. Save only that sheet as CSV UTF-8 (comma-delimited). 3. In Jota &gt; Content &gt; Import from CSV, upload it, choose any shared defaults, fix preview errors, then import.</x:v>
+        <x:v>1. Add one content item per row on Content Import. 2. Export only that sheet as CSV UTF-8. 3. In Jota, upload the CSV, choose one client, review the preview, and import.</x:v>
       </x:c>
       <x:c r="B3" s="14"/>
       <x:c r="C3" s="14"/>
@@ -668,7 +661,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="str">
-        <x:v>Optional AI prompt to copy</x:v>
+        <x:v>Optional prompt for an image or content plan</x:v>
       </x:c>
       <x:c r="B5" s="16"/>
       <x:c r="C5" s="16"/>
@@ -676,10 +669,9 @@
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="34" t="str">
-        <x:v>Convert the content plan I paste after this prompt into a UTF-8 CSV for Jota. Copy the exact 17 headers from the Content Import sheet in the same order. Make one row per real content item.
-Use only source facts. Do not invent posts, clients, campaigns, platforms, formats, dates, assigned people, workflow statuses, or external client approval. Use exact active Jota names only when I supply them. Repeat the client name in Client / account for every row, even when all rows share one client. Fill Assigned creator / editor with the exact active member name when a supervisor or admin assigns content. Leave Campaign blank for General / Ongoing.
-Every row needs Content title, Platform, and Format. Ask me about missing required details before making the CSV. Use YYYY-MM-DD: Publish date is the posting date, Work date is when production starts, and Deadline is when work is due. Leave unknown optional cells empty; a blank Status becomes Planned.
-Quote commas, quotation marks, and line breaks correctly. Exclude the AI Guide, sample record, formulas, and explanations. Return only the CSV.</x:v>
+        <x:v>Read the calendar image or content plan I provide and make a UTF-8 CSV with exactly these headers: Content title,Platform,Format,Publish date,Work date,Deadline,Brief / caption. Make one row per real content item.
+Copy only details visible or stated. Do not invent titles, platforms, formats, dates, or captions. Use YYYY-MM-DD for dates; leave unknown optional dates and captions empty. Ask me about missing Content title, Platform, or Format before producing the CSV.
+Do not add client, campaign, account manager, video editor, status, or approval columns. Jota handles client and assignment separately. Quote CSV commas and line breaks correctly. Return only CSV, without an example row or explanation.</x:v>
       </x:c>
       <x:c r="B6" s="35"/>
       <x:c r="C6" s="35"/>
@@ -699,219 +691,185 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="16" t="str">
-        <x:v>Import rules</x:v>
+        <x:v>What to fill in</x:v>
       </x:c>
       <x:c r="B10" s="16"/>
       <x:c r="C10" s="16"/>
       <x:c r="D10" s="16"/>
     </x:row>
-    <x:row r="11" ht="32" customHeight="1">
+    <x:row r="11" ht="40" customHeight="1">
       <x:c r="A11" s="46" t="str">
-        <x:v>Client / account</x:v>
+        <x:v>Content title</x:v>
       </x:c>
       <x:c r="B11" s="47" t="str">
-        <x:v>Fill every row with an exact active Jota client name, even when all rows belong to the same client.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="32" customHeight="1">
+        <x:v>Required. One actual post or creative piece per row; use a clear title.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
       <x:c r="A12" s="48" t="str">
-        <x:v>Campaign</x:v>
+        <x:v>Platform and Format</x:v>
       </x:c>
       <x:c r="B12" s="49" t="str">
-        <x:v>Optional. Use the exact active campaign name for that client. Leave blank to use General / Ongoing.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="46" customHeight="1">
+        <x:v>Required for each row. Examples: Instagram + Reel, or Facebook + Static image. Format tells Jota whether content is video or static.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="40" customHeight="1">
       <x:c r="A13" s="48" t="str">
-        <x:v>Required content fields</x:v>
+        <x:v>Publish date</x:v>
       </x:c>
       <x:c r="B13" s="49" t="str">
-        <x:v>Each row needs Content title, Platform, and Format. Supervisors/admins must also enter the exact active Assigned creator / editor name for that client.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="32" customHeight="1">
+        <x:v>Optional planned posting date. Use YYYY-MM-DD; leave blank when unscheduled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="40" customHeight="1">
       <x:c r="A14" s="48" t="str">
-        <x:v>Dates</x:v>
+        <x:v>Work date</x:v>
       </x:c>
       <x:c r="B14" s="49" t="str">
-        <x:v>Dates are optional. Use YYYY-MM-DD with a year: Work date starts production, Deadline is when work is due, and Publish date is the scheduled posting date.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="32" customHeight="1">
+        <x:v>Optional date production starts. Use YYYY-MM-DD.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="40" customHeight="1">
       <x:c r="A15" s="48" t="str">
-        <x:v>Status</x:v>
+        <x:v>Deadline</x:v>
       </x:c>
       <x:c r="B15" s="49" t="str">
-        <x:v>Optional. Supported values include Idea, Planned, In Production, For Review, Revision Requested, Waiting Client, Scheduled, Published, Rejected, and Cancelled. Blank defaults to Planned.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+        <x:v>Optional date the work is due. Use YYYY-MM-DD.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="40" customHeight="1">
       <x:c r="A16" s="48" t="str">
-        <x:v>Client approval</x:v>
+        <x:v>Brief / caption</x:v>
       </x:c>
       <x:c r="B16" s="49" t="str">
-        <x:v>Optional. Record Pending, Approved, Revision Requested, or Rejected only after a real response through your external client channel. Do not infer approval from status.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32" customHeight="1">
+        <x:v>Optional short instruction or draft caption. Leave unknown details blank.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="40" customHeight="1">
       <x:c r="A17" s="48" t="str">
-        <x:v>Revision count</x:v>
+        <x:v>Client and account manager</x:v>
       </x:c>
       <x:c r="B17" s="49" t="str">
-        <x:v>Optional whole number from 0 to 10,000. Blank defaults to 0.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="32" customHeight="1">
+        <x:v>Do not put these in the file. Choose one client in Jota. Account-manager imports assign the creator/editor to the signed-in manager; supervisors/admins choose a client member.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="40" customHeight="1">
       <x:c r="A18" s="48" t="str">
-        <x:v>CSV export</x:v>
+        <x:v>Video editor</x:v>
       </x:c>
       <x:c r="B18" s="49" t="str">
-        <x:v>Save only the Content Import sheet as CSV UTF-8 (comma-delimited), not XLSX. Keep headers in row 1; do not include this guide or its sample record.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="38" customHeight="1">
+        <x:v>The current import screen has no bulk video-editor picker. After importing, edit each video content card to choose its editor. Do not assume the client-level editor was assigned automatically.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="40" customHeight="1">
       <x:c r="A19" s="50" t="str">
-        <x:v>Import limit</x:v>
+        <x:v>Export and limits</x:v>
       </x:c>
       <x:c r="B19" s="51" t="str">
-        <x:v>The CSV must be 1 MB or smaller and contain at most 250 content rows. Check the preview: fix invalid rows before importing; duplicates are skipped.</x:v>
+        <x:v>Export only Content Import as CSV UTF-8, not XLSX. Maximum 1 MB and 250 rows. New items start as Planned; preview errors must be fixed, and duplicates are skipped.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="53" t="str">
-        <x:v>Sample record (reference only; do not import)</x:v>
+        <x:v>Example values (reference only; do not import)</x:v>
       </x:c>
       <x:c r="B21" s="53"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="55" t="str">
-        <x:v>Client / account</x:v>
+        <x:v>Content title</x:v>
       </x:c>
       <x:c r="B22" s="61" t="str">
-        <x:v>Replace with an exact active client name</x:v>
+        <x:v>Behind the scenes: preparing the new menu</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
       <x:c r="A23" s="57" t="str">
-        <x:v>Campaign</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="B23" s="62" t="str">
-        <x:v>Existing campaign name or blank</x:v>
+        <x:v>Instagram</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="57" t="str">
-        <x:v>Content title</x:v>
+        <x:v>Format</x:v>
       </x:c>
       <x:c r="B24" s="58" t="str">
-        <x:v>Behind the scenes: preparing the new menu</x:v>
+        <x:v>Reel</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26" customHeight="1">
       <x:c r="A25" s="57" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Publish date</x:v>
       </x:c>
       <x:c r="B25" s="58" t="str">
-        <x:v>Instagram</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="26" customHeight="1">
       <x:c r="A26" s="57" t="str">
-        <x:v>Format</x:v>
+        <x:v>Work date</x:v>
       </x:c>
       <x:c r="B26" s="58" t="str">
-        <x:v>Reel</x:v>
+        <x:v>2026-10-27</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26" customHeight="1">
       <x:c r="A27" s="57" t="str">
-        <x:v>Status</x:v>
+        <x:v>Deadline</x:v>
       </x:c>
       <x:c r="B27" s="58" t="str">
-        <x:v>Planned</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26" customHeight="1">
       <x:c r="A28" s="57" t="str">
-        <x:v>Work date</x:v>
+        <x:v>Brief / caption</x:v>
       </x:c>
       <x:c r="B28" s="58" t="str">
-        <x:v>2026-10-19</x:v>
+        <x:v>Show the team preparing the new menu.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="26" customHeight="1">
-      <x:c r="A29" s="57" t="str">
-        <x:v>Deadline</x:v>
-      </x:c>
-      <x:c r="B29" s="58" t="str">
-        <x:v>2026-10-21</x:v>
-      </x:c>
+      <x:c r="A29"/>
+      <x:c r="B29"/>
     </x:row>
     <x:row r="30" ht="26" customHeight="1">
-      <x:c r="A30" s="57" t="str">
-        <x:v>Publish date</x:v>
-      </x:c>
-      <x:c r="B30" s="58" t="str">
-        <x:v>2026-10-22</x:v>
-      </x:c>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
     </x:row>
     <x:row r="31" ht="26" customHeight="1">
-      <x:c r="A31" s="57" t="str">
-        <x:v>Client approval</x:v>
-      </x:c>
-      <x:c r="B31" s="58" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
+      <x:c r="A31"/>
+      <x:c r="B31"/>
     </x:row>
     <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="57" t="str">
-        <x:v>Client issues</x:v>
-      </x:c>
-      <x:c r="B32" s="58" t="str"/>
+      <x:c r="A32"/>
+      <x:c r="B32"/>
     </x:row>
     <x:row r="33" ht="26" customHeight="1">
-      <x:c r="A33" s="57" t="str">
-        <x:v>Revision count</x:v>
-      </x:c>
-      <x:c r="B33" s="58" t="str">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="A33"/>
+      <x:c r="B33"/>
     </x:row>
     <x:row r="34" ht="26" customHeight="1">
-      <x:c r="A34" s="57" t="str">
-        <x:v>Notes / comments</x:v>
-      </x:c>
-      <x:c r="B34" s="58" t="str"/>
+      <x:c r="A34"/>
+      <x:c r="B34"/>
     </x:row>
     <x:row r="35" ht="26" customHeight="1">
-      <x:c r="A35" s="57" t="str">
-        <x:v>Brief / caption</x:v>
-      </x:c>
-      <x:c r="B35" s="58" t="str">
-        <x:v>Show a quick behind-the-scenes look at preparation.</x:v>
-      </x:c>
+      <x:c r="A35"/>
+      <x:c r="B35"/>
     </x:row>
     <x:row r="36" ht="26" customHeight="1">
-      <x:c r="A36" s="57" t="str">
-        <x:v>Next action</x:v>
-      </x:c>
-      <x:c r="B36" s="58" t="str">
-        <x:v>Prepare first draft</x:v>
-      </x:c>
+      <x:c r="A36"/>
+      <x:c r="B36"/>
     </x:row>
     <x:row r="37" ht="26" customHeight="1">
-      <x:c r="A37" s="57" t="str">
-        <x:v>Revision feedback</x:v>
-      </x:c>
-      <x:c r="B37" s="58" t="str"/>
+      <x:c r="A37"/>
+      <x:c r="B37"/>
     </x:row>
     <x:row r="38" ht="26" customHeight="1">
-      <x:c r="A38" s="59" t="str">
-        <x:v>Assigned creator / editor</x:v>
-      </x:c>
-      <x:c r="B38" s="63" t="str">
-        <x:v>Exact active client member name or blank</x:v>
-      </x:c>
+      <x:c r="A38"/>
+      <x:c r="B38"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Enable supervisor content ownership and completed content filter
</commit_message>
<xml_diff>
--- a/public/content-import-template.xlsx
+++ b/public/content-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Import" sheetId="1" r:id="R72329bf4122645ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Guide" sheetId="2" r:id="Rd037121c4a76421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Import" sheetId="1" r:id="Rb37ea0a156274a4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Guide" sheetId="2" r:id="R2fa2f480a1b84a6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -750,7 +750,7 @@
         <x:v>Client and account manager</x:v>
       </x:c>
       <x:c r="B17" s="49" t="str">
-        <x:v>Do not put these in the file. Choose one client in Jota. Account-manager imports assign the creator/editor to the signed-in manager; supervisors/admins choose a client member.</x:v>
+        <x:v>Do not put these in the file. Choose one client in Jota. Account managers and supervisors default to themselves as creator/editor when available; they can choose another eligible person.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -758,7 +758,7 @@
         <x:v>Video editor</x:v>
       </x:c>
       <x:c r="B18" s="49" t="str">
-        <x:v>The current import screen has no bulk video-editor picker. After importing, edit each video content card to choose its editor. Do not assume the client-level editor was assigned automatically.</x:v>
+        <x:v>If the CSV includes video rows, you can optionally choose the client's designated video editor on the import screen. Video rows use that editor; static rows keep the selected creator.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="40" customHeight="1">

</xml_diff>